<commit_message>
trend screener update 2026-09-03 14:47 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3511,12 +3511,12 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>0688.HK</t>
+          <t>1908.HK</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>中国海外发展</t>
+          <t>建发国际集团</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -3534,18 +3534,18 @@
         <v>4</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>13.17</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>1908.HK</t>
+          <t>0688.HK</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>建发国际集团</t>
+          <t>中国海外发展</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -3563,7 +3563,7 @@
         <v>4</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>12.8</v>
+        <v>13.17</v>
       </c>
     </row>
     <row r="36">
@@ -3712,72 +3712,72 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>9999.HK</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>网易-S</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr"/>
+      <c r="F41" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>9618.HK</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>京东集团-SW</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>B·EXIT 🔴</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="n">
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G41" s="3" t="n">
+      <c r="G42" s="3" t="n">
         <v>106.9</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>9888.HK</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>百度集团-SW</t>
-        </is>
-      </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr"/>
-      <c r="F42" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>91.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>9999.HK</t>
+          <t>9888.HK</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>网易-S</t>
+          <t>百度集团-SW</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
@@ -3795,7 +3795,7 @@
         <v>3</v>
       </c>
       <c r="G43" s="12" t="n">
-        <v>183</v>
+        <v>91.5</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
trend screener update 2026-09-03 16:29 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3511,12 +3511,12 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>1908.HK</t>
+          <t>0688.HK</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>建发国际集团</t>
+          <t>中国海外发展</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -3534,18 +3534,18 @@
         <v>4</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>12.8</v>
+        <v>13.17</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>0688.HK</t>
+          <t>0817.HK</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>中国海外发展</t>
+          <t>中国金茂</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -3563,18 +3563,18 @@
         <v>4</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>13.17</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>0817.HK</t>
+          <t>1908.HK</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>中国金茂</t>
+          <t>建发国际集团</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -3592,7 +3592,7 @@
         <v>4</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>1.35</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
trend screener update 2026-09-09 00:42 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -985,366 +985,366 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>0285.HK</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>比亚迪电子</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>3993.HK</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>洛阳钼业</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>工业金属</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>16.943</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>0136.HK</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>中国儒意</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>媒体及娱乐</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1.372</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>-3.65</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>-6.61</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>1138.HK</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>中远海能</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>交运</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>16.852</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>9699.HK</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>顺丰同城</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>交运</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>SOS-C</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>8.426</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>-3.97</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>0999.HK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>小菜园</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>旅游及消闲设施</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>SOS-C</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>7.659</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>-3.28</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>6078.HK</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>海吉亚医疗</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>其他医疗保健</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>SOS-C</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>10.275</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>-2.78</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>0354.HK</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>中国软件国际</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>消费电子</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>软件服务</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>25.52</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>25.342</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>7.15</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>-4.13</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>3993.HK</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>洛阳钼业</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>工业金属</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>SOS-C</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>3.815</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>3.883</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>-4.75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2799.HK</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>中信金融资产</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>其他金融</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>17.61</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>16.943</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>0136.HK</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>中国儒意</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>媒体及娱乐</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>1.372</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>-3.65</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>-6.61</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>1138.HK</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>中远海能</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>交运</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>17.99</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>16.852</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>10.38</v>
-      </c>
-      <c r="J14" s="8" t="n">
-        <v>4.34</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>9699.HK</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>顺丰同城</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>交运</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>8.426</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>-3.97</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>0999.HK</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>小菜园</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>旅游及消闲设施</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>SOS-C</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>8.130000000000001</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>7.659</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>-3.28</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>6078.HK</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>海吉亚医疗</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>其他医疗保健</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>SOS-C</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>10.44</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>10.275</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>5.16</v>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>-2.78</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>0354.HK</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>中国软件国际</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>软件服务</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>SOS-C</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>3.815</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>3.883</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>8.83</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>-4.75</v>
+      <c r="G18" s="9" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>-5.08</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>2799.HK</t>
+          <t>3958.HK</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>中信金融资产</t>
+          <t>东方证券</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1368,235 +1368,191 @@
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>0.655</v>
+        <v>5.8</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.646</v>
+        <v>5.855</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>7.58</v>
+        <v>4.84</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-5.08</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>3958.HK</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>东方证券</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>其他金融</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>1797.HK</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>东方甄选</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>零售</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G20" s="9" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>5.855</v>
-      </c>
-      <c r="I20" s="9" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>-2.31</v>
+      <c r="G20" s="10" t="n">
+        <v>26.62</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>25.544</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>0.47</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>1797.HK</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>东方甄选</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>零售</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>1357.HK</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>美图公司</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>媒体及娱乐</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G21" s="10" t="n">
-        <v>26.62</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>25.544</v>
-      </c>
-      <c r="I21" s="10" t="n">
-        <v>20.12</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>0.47</v>
+      <c r="G21" s="7" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>4.649</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>-6.61</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>1357.HK</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>美图公司</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>媒体及娱乐</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2688.HK</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>新奥能源</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>公共事业</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G22" s="7" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="H22" s="7" t="n">
-        <v>4.649</v>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>6.43</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>-6.61</v>
+      <c r="G22" s="11" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>49.29</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="J22" s="11" t="n">
+        <v>-2.8</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>2688.HK</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>新奥能源</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Utilities</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>公共事业</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>3668.HK</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>兖煤澳大利亚</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>能源</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="H23" s="11" t="n">
-        <v>49.29</v>
-      </c>
-      <c r="I23" s="11" t="n">
-        <v>4.08</v>
-      </c>
-      <c r="J23" s="11" t="n">
-        <v>-2.8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>3668.HK</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>兖煤澳大利亚</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>能源</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>SOS-C</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="n">
+      <c r="G23" s="8" t="n">
         <v>36.22</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H23" s="8" t="n">
         <v>34.253</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I23" s="8" t="n">
         <v>6.88</v>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J23" s="8" t="n">
         <v>1.73</v>
       </c>
     </row>
@@ -3089,12 +3045,12 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>0688.HK</t>
+          <t>0960.HK</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>中国海外发展</t>
+          <t>龙湖集团</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -3112,18 +3068,18 @@
         <v>2</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>13.01</v>
+        <v>6.225</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>0960.HK</t>
+          <t>1908.HK</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>龙湖集团</t>
+          <t>建发国际集团</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -3141,18 +3097,18 @@
         <v>2</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>6.225</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>1908.HK</t>
+          <t>0688.HK</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>建发国际集团</t>
+          <t>中国海外发展</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
@@ -3170,7 +3126,7 @@
         <v>2</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>12.7</v>
+        <v>13.01</v>
       </c>
     </row>
     <row r="31">
@@ -3408,12 +3364,12 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>0168.HK</t>
+          <t>1876.HK</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>青岛啤酒股份</t>
+          <t>百威亚太</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -3431,18 +3387,18 @@
         <v>2</v>
       </c>
       <c r="G39" s="10" t="n">
-        <v>41.46</v>
+        <v>6.115</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>1876.HK</t>
+          <t>0168.HK</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>百威亚太</t>
+          <t>青岛啤酒股份</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -3460,7 +3416,7 @@
         <v>2</v>
       </c>
       <c r="G40" s="10" t="n">
-        <v>6.115</v>
+        <v>41.46</v>
       </c>
     </row>
     <row r="41">
@@ -4630,7 +4586,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>扫描日期：2026-09-08</t>
+          <t>扫描日期：2026-09-09</t>
         </is>
       </c>
     </row>

</xml_diff>